<commit_message>
fix: parse empty receipt fields correctly; record live-verified defects
Verified against demoblaze.com: selectors, API contracts and BUG-01..05.
Claude-Session: https://claude.ai/code/session_01HEwwY9GdDTh7kNhnnohezE
</commit_message>
<xml_diff>
--- a/test-cases/DemoBlaze_TestCases.xlsx
+++ b/test-cases/DemoBlaze_TestCases.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="536">
   <si>
     <t xml:space="preserve">DemoBlaze — Test Case Suite (Login, Cart, Place Order)</t>
   </si>
@@ -1622,7 +1622,7 @@
     <t xml:space="preserve">Month is one less (JS getMonth() is zero-based); e.g. October shows as 9</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmed in source (cart.js)</t>
+    <t xml:space="preserve">Verified live on demoblaze.com (13 Oct 2026): receipt showed 13/9/2026 in October</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-02</t>
@@ -1643,7 +1643,7 @@
     <t xml:space="preserve">Receipt is shown with Amount 0</t>
   </si>
   <si>
-    <t xml:space="preserve">To confirm on first CI run</t>
+    <t xml:space="preserve">Verified live on demoblaze.com (13 Oct 2026): receipt with Amount 0 USD</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-03</t>
@@ -1661,7 +1661,7 @@
     <t xml:space="preserve">Order accepted</t>
   </si>
   <si>
-    <t xml:space="preserve">Only emptiness is checked (cart.js)</t>
+    <t xml:space="preserve">Verified live on demoblaze.com (13 Oct 2026): card 'not-a-card' accepted</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-04</t>
@@ -1679,6 +1679,9 @@
     <t xml:space="preserve">Treated as empty</t>
   </si>
   <si>
+    <t xml:space="preserve">Verified live on demoblaze.com (13 Oct 2026): receipt shows empty 'Name:'</t>
+  </si>
+  <si>
     <t xml:space="preserve">BUG-05</t>
   </si>
   <si>
@@ -1697,6 +1700,9 @@
     <t xml:space="preserve">Full number displayed</t>
   </si>
   <si>
+    <t xml:space="preserve">Verified live on demoblaze.com (13 Oct 2026): full 16-digit number shown</t>
+  </si>
+  <si>
     <t xml:space="preserve">BUG-06</t>
   </si>
   <si>
@@ -1715,7 +1721,7 @@
     <t xml:space="preserve">TC-CART-001 / 004</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmed in source (prod.js)</t>
+    <t xml:space="preserve">Logged-in alert 'Product added.' verified live; guest variant from prod.js</t>
   </si>
   <si>
     <t xml:space="preserve">OBS-01</t>
@@ -6373,7 +6379,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
         <v>487</v>
       </c>
@@ -6402,7 +6408,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
         <v>494</v>
       </c>
@@ -6431,7 +6437,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>501</v>
       </c>
@@ -6460,7 +6466,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>507</v>
       </c>
@@ -6486,94 +6492,94 @@
         <v>349</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>489</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>385</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>509</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>